<commit_message>
Updated models and monitor
</commit_message>
<xml_diff>
--- a/financial_models/Macro_Monitor.xlsx
+++ b/financial_models/Macro_Monitor.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerry\PycharmProjects\Invest_Proc_v4\financial_models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE33E23-7707-408F-8F21-4F075F8358E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D0397B3-B2D9-424F-876C-AC256E6A8D47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="33720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Market_Yield" sheetId="2" r:id="rId1"/>
+    <sheet name="Framework" sheetId="10" r:id="rId1"/>
     <sheet name="Forex" sheetId="9" r:id="rId2"/>
     <sheet name="Equity_Indices" sheetId="8" r:id="rId3"/>
     <sheet name="Economies" sheetId="4" r:id="rId4"/>
     <sheet name="Commodities" sheetId="5" r:id="rId5"/>
     <sheet name="Real_Estate" sheetId="6" r:id="rId6"/>
+    <sheet name="Market_Yield" sheetId="2" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="209">
   <si>
     <t>China</t>
   </si>
@@ -641,10 +642,6 @@
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
   <si>
-    <t>Market Yields:</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
     <t>Notes</t>
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
@@ -653,10 +650,6 @@
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
   <si>
-    <t>Valuation Model Assumptions</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
     <t>CRB Commodity Index</t>
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
@@ -669,22 +662,6 @@
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
   <si>
-    <t>Target Annual Return</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>Base Cost of Equity</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>China</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>HK</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
     <t>https://tradingeconomics.com/hong-kong/government-bond-yield</t>
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
@@ -709,18 +686,6 @@
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
   <si>
-    <t>Prime Rate</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>Risk Premium</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>Riskfree rate</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
     <t>https://tradingeconomics.com/china/government-bond-yield</t>
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
@@ -733,10 +698,6 @@
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
   <si>
-    <t>Benchmarket Return:</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
     <t>https://awealthofcommonsense.com/2025/01/historical-returns-for-stocks-bonds-cash-real-estate-and-gold/</t>
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
@@ -745,35 +706,212 @@
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
   <si>
-    <t>Stocks</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>Small caps</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>Bonds</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>Cash</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>Gold</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>Real estate</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>US (1928-2024)</t>
-    <phoneticPr fontId="11" type="noConversion"/>
-  </si>
-  <si>
-    <t>Benchmark for stocks</t>
+    <t>Sector Analysis</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>Country/Region Analysis</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>Use PEST analysis</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>Porter's Five Forces</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>Company Analysis</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>5W2H</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>方法</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>SWOT</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>第一：了解行业现状</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>产业链图</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>产业分赃链图</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>市场规模预估法实现</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>第二：分析行业动能</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>外部动能</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DengXian"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>内部动能</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DengXian"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>竞争壁垒</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DengXian"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>行业周期</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>第三：推测行业变化</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DengXian"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>竞品分析</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>第四：找出行业带给自身的机会</t>
+    </r>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>商业模式画布</t>
+    </r>
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
 </sst>
@@ -781,9 +919,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="&quot;for &quot;0&quot; Yrs&quot;"/>
-  </numFmts>
   <fonts count="19">
     <font>
       <sz val="11"/>
@@ -906,15 +1041,17 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
+      <color theme="1"/>
+      <name val="Microsoft YaHei"/>
       <family val="1"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Times New Roman"/>
+      <color theme="1"/>
+      <name val="DengXian"/>
       <family val="1"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="7">
@@ -955,7 +1092,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1037,27 +1174,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1165,33 +1287,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="176" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="10" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1472,286 +1568,104 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A061C73F-1F33-4614-90A5-D5D9D7C58056}">
-  <dimension ref="A2:E36"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEDB0449-8591-42B7-B720-6314A45F3007}">
+  <dimension ref="A2:F15"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="1" max="1" width="2.46484375" style="7" customWidth="1"/>
-    <col min="2" max="2" width="30.19921875" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="15.59765625" style="7" customWidth="1"/>
-    <col min="6" max="16384" width="8.796875" style="7"/>
+    <col min="1" max="1" width="2.59765625" style="7" customWidth="1"/>
+    <col min="2" max="2" width="37.265625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" style="7" customWidth="1"/>
+    <col min="4" max="5" width="18.3984375" style="7" customWidth="1"/>
+    <col min="6" max="6" width="19.73046875" style="7" customWidth="1"/>
+    <col min="7" max="16384" width="9.06640625" style="7"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="15">
+    <row r="2" spans="1:6" ht="15">
       <c r="A2" s="3"/>
       <c r="B2" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="4"/>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="4"/>
-      <c r="B3" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C3" s="45">
-        <v>0.2</v>
-      </c>
-      <c r="D3" s="48">
-        <v>3</v>
-      </c>
-      <c r="E3" s="46"/>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="4"/>
+        <v>190</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="B4" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="C4" s="49">
-        <f>MAX(8%,C8:D10)</f>
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="15">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15">
       <c r="A6" s="3"/>
       <c r="B6" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="4"/>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="C7" s="15" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15">
+      <c r="B8" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15">
+      <c r="B9" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15">
+      <c r="B10" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15">
+      <c r="B11" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15">
+      <c r="A13" s="3"/>
+      <c r="B13" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="B14" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="B8" s="50" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="51">
-        <v>4.2500000000000003E-2</v>
-      </c>
-      <c r="D8" s="51">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="E8" s="52">
-        <f>D8-C8</f>
-        <v>3.2499999999999994E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="B9" s="50" t="s">
-        <v>182</v>
-      </c>
-      <c r="C9" s="51">
-        <v>1.9E-2</v>
-      </c>
-      <c r="D9" s="51">
-        <v>3.1E-2</v>
-      </c>
-      <c r="E9" s="52">
-        <f>D9-C9</f>
-        <v>1.2E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="B10" s="50" t="s">
-        <v>183</v>
-      </c>
-      <c r="C10" s="51">
-        <v>3.4500000000000003E-2</v>
-      </c>
-      <c r="D10" s="51">
-        <v>5.2499999999999998E-2</v>
-      </c>
-      <c r="E10" s="52">
-        <f>D10-C10</f>
-        <v>1.7999999999999995E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="15">
-      <c r="A12" s="3"/>
-      <c r="B12" s="2" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="C13" s="15" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="B14" s="53" t="s">
-        <v>199</v>
-      </c>
-      <c r="C14" s="51">
-        <v>9.9400000000000002E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="B15" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="C15" s="51">
-        <v>0.1174</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="B16" s="53" t="s">
-        <v>201</v>
-      </c>
-      <c r="C16" s="51">
-        <v>3.4500000000000003E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="B17" s="53" t="s">
-        <v>202</v>
-      </c>
-      <c r="C17" s="51">
-        <v>3.3099999999999997E-2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="B18" s="53" t="s">
-        <v>204</v>
-      </c>
-      <c r="C18" s="51">
-        <v>4.2299999999999997E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="B19" s="53" t="s">
-        <v>203</v>
-      </c>
-      <c r="C19" s="51">
-        <v>5.1200000000000002E-2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="B20" s="54" t="s">
-        <v>206</v>
-      </c>
-      <c r="C20" s="55">
-        <f>MAX(C4,C14:C19)</f>
-        <v>0.1174</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="15">
-      <c r="A23" s="3"/>
-      <c r="B23" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="47"/>
-      <c r="E23" s="4"/>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="B24" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="B25" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="C25" s="16" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="B26" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="C27" s="16"/>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="B28" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="B29" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="C30" s="16"/>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="B31" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="C31" s="16" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5">
-      <c r="B32" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="C32" s="16" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="33" spans="2:3">
-      <c r="C33" s="16"/>
-    </row>
-    <row r="34" spans="2:3">
-      <c r="B34" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="C34" s="16" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="36" spans="2:3">
-      <c r="B36" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="C36" s="16" t="s">
-        <v>197</v>
+    </row>
+    <row r="15" spans="1:6" ht="15">
+      <c r="B15" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="11" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="C28" r:id="rId1" xr:uid="{45D5643F-FA1A-3C48-B2D9-4B6082295A37}"/>
-    <hyperlink ref="C24" r:id="rId2" xr:uid="{8FF27AF7-25A6-F443-A0E6-DAC1AFC8FB4A}"/>
-    <hyperlink ref="C34" r:id="rId3" xr:uid="{E414D4D1-755D-2A43-AB81-B4A0517E9107}"/>
-    <hyperlink ref="C25" r:id="rId4" xr:uid="{BD25C893-4B01-48BE-AB6E-FA9F70DB6325}"/>
-    <hyperlink ref="C29" r:id="rId5" xr:uid="{01B23463-056A-45A3-AFE5-8FCBFF68216B}"/>
-    <hyperlink ref="C31" r:id="rId6" xr:uid="{CA446899-0FC4-4E1D-9FA6-827A1A2C6101}"/>
-    <hyperlink ref="C32" r:id="rId7" xr:uid="{2A60B260-D4EE-4AB2-B4D5-2C97E9E3A2EB}"/>
-    <hyperlink ref="C26" r:id="rId8" xr:uid="{7EACBB86-54AE-4C08-9D45-813ABBBD2BC8}"/>
-    <hyperlink ref="C36" r:id="rId9" xr:uid="{30137619-E054-41EB-9359-F9138F1700F2}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId10"/>
 </worksheet>
 </file>
 
@@ -1768,10 +1682,10 @@
     <row r="2" spans="1:5" ht="15">
       <c r="A2" s="3"/>
       <c r="B2" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C2" s="4"/>
-      <c r="D2" s="47"/>
+      <c r="D2" s="45"/>
       <c r="E2" s="4"/>
     </row>
     <row r="3" spans="1:5">
@@ -2995,12 +2909,12 @@
     <row r="2" spans="1:3" ht="15">
       <c r="A2" s="3"/>
       <c r="B2" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="B3" s="12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C3" s="13" t="s">
         <v>128</v>
@@ -3098,7 +3012,7 @@
     <row r="2" spans="1:4" ht="15">
       <c r="A2" s="3"/>
       <c r="B2" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -3149,4 +3063,123 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A061C73F-1F33-4614-90A5-D5D9D7C58056}">
+  <dimension ref="A2:E15"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.9"/>
+  <cols>
+    <col min="1" max="1" width="2.46484375" style="7" customWidth="1"/>
+    <col min="2" max="2" width="30.19921875" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="15.59765625" style="7" customWidth="1"/>
+    <col min="6" max="16384" width="8.796875" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:5" ht="15">
+      <c r="A2" s="3"/>
+      <c r="B2" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C2" s="4"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="4"/>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="B3" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="B4" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="B5" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="C6" s="16"/>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="B7" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="B8" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="C9" s="16"/>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="B10" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="B11" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="C12" s="16"/>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="B13" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="B15" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>187</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="11" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C7" r:id="rId1" xr:uid="{45D5643F-FA1A-3C48-B2D9-4B6082295A37}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{8FF27AF7-25A6-F443-A0E6-DAC1AFC8FB4A}"/>
+    <hyperlink ref="C13" r:id="rId3" xr:uid="{E414D4D1-755D-2A43-AB81-B4A0517E9107}"/>
+    <hyperlink ref="C4" r:id="rId4" xr:uid="{BD25C893-4B01-48BE-AB6E-FA9F70DB6325}"/>
+    <hyperlink ref="C8" r:id="rId5" xr:uid="{01B23463-056A-45A3-AFE5-8FCBFF68216B}"/>
+    <hyperlink ref="C10" r:id="rId6" xr:uid="{CA446899-0FC4-4E1D-9FA6-827A1A2C6101}"/>
+    <hyperlink ref="C11" r:id="rId7" xr:uid="{2A60B260-D4EE-4AB2-B4D5-2C97E9E3A2EB}"/>
+    <hyperlink ref="C5" r:id="rId8" xr:uid="{7EACBB86-54AE-4C08-9D45-813ABBBD2BC8}"/>
+    <hyperlink ref="C15" r:id="rId9" xr:uid="{30137619-E054-41EB-9359-F9138F1700F2}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId10"/>
+</worksheet>
 </file>
</xml_diff>